<commit_message>
Added gunicorn for Render deployment
</commit_message>
<xml_diff>
--- a/cv_analyzer/data/applicants.xlsx
+++ b/cv_analyzer/data/applicants.xlsx
@@ -15605,22 +15605,22 @@
         <v>5</v>
       </c>
       <c r="AN77" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO77" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="AP77" t="n">
         <v>30</v>
       </c>
       <c r="AQ77" t="n">
-        <v>54</v>
+        <v>47.8</v>
       </c>
       <c r="AR77" t="n">
         <v>100</v>
       </c>
       <c r="AS77" t="n">
-        <v>54</v>
+        <v>47.8</v>
       </c>
       <c r="AT77" t="inlineStr">
         <is>
@@ -15804,7 +15804,7 @@
         <v>5</v>
       </c>
       <c r="AN78" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AO78" t="n">
         <v>28</v>
@@ -15813,13 +15813,13 @@
         <v>30</v>
       </c>
       <c r="AQ78" t="n">
-        <v>56.6</v>
+        <v>54.2</v>
       </c>
       <c r="AR78" t="n">
         <v>100</v>
       </c>
       <c r="AS78" t="n">
-        <v>56.6</v>
+        <v>54.2</v>
       </c>
       <c r="AT78" t="inlineStr">
         <is>
@@ -16003,22 +16003,22 @@
         <v>5</v>
       </c>
       <c r="AN79" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AO79" t="n">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="AP79" t="n">
         <v>30</v>
       </c>
       <c r="AQ79" t="n">
-        <v>67.59999999999999</v>
+        <v>58</v>
       </c>
       <c r="AR79" t="n">
         <v>100</v>
       </c>
       <c r="AS79" t="n">
-        <v>67.59999999999999</v>
+        <v>58</v>
       </c>
       <c r="AT79" t="inlineStr">
         <is>
@@ -16206,22 +16206,22 @@
         <v>5</v>
       </c>
       <c r="AN80" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO80" t="n">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="AP80" t="n">
         <v>30</v>
       </c>
       <c r="AQ80" t="n">
-        <v>85.2</v>
+        <v>78.2</v>
       </c>
       <c r="AR80" t="n">
         <v>100</v>
       </c>
       <c r="AS80" t="n">
-        <v>85.2</v>
+        <v>78.2</v>
       </c>
       <c r="AT80" t="inlineStr">
         <is>
@@ -16409,22 +16409,22 @@
         <v>5</v>
       </c>
       <c r="AN81" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO81" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="AP81" t="n">
         <v>30</v>
       </c>
       <c r="AQ81" t="n">
-        <v>69.59999999999999</v>
+        <v>61</v>
       </c>
       <c r="AR81" t="n">
         <v>100</v>
       </c>
       <c r="AS81" t="n">
-        <v>69.59999999999999</v>
+        <v>61</v>
       </c>
       <c r="AT81" t="inlineStr">
         <is>
@@ -16608,22 +16608,22 @@
         <v>5</v>
       </c>
       <c r="AN82" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AO82" t="n">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="AP82" t="n">
         <v>30</v>
       </c>
       <c r="AQ82" t="n">
-        <v>85.40000000000001</v>
+        <v>78.2</v>
       </c>
       <c r="AR82" t="n">
         <v>100</v>
       </c>
       <c r="AS82" t="n">
-        <v>85.40000000000001</v>
+        <v>78.2</v>
       </c>
       <c r="AT82" t="inlineStr">
         <is>
@@ -16810,19 +16810,19 @@
         <v>50</v>
       </c>
       <c r="AO83" t="n">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="AP83" t="n">
         <v>30</v>
       </c>
       <c r="AQ83" t="n">
-        <v>53.8</v>
+        <v>49</v>
       </c>
       <c r="AR83" t="n">
         <v>100</v>
       </c>
       <c r="AS83" t="n">
-        <v>53.8</v>
+        <v>49</v>
       </c>
       <c r="AT83" t="inlineStr">
         <is>
@@ -17006,22 +17006,22 @@
         <v>5</v>
       </c>
       <c r="AN84" t="n">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="AO84" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="AP84" t="n">
         <v>30</v>
       </c>
       <c r="AQ84" t="n">
-        <v>77.59999999999999</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="AR84" t="n">
         <v>100</v>
       </c>
       <c r="AS84" t="n">
-        <v>77.59999999999999</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="AT84" t="inlineStr">
         <is>
@@ -17205,22 +17205,22 @@
         <v>5</v>
       </c>
       <c r="AN85" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO85" t="n">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="AP85" t="n">
         <v>30</v>
       </c>
       <c r="AQ85" t="n">
-        <v>84.8</v>
+        <v>78.2</v>
       </c>
       <c r="AR85" t="n">
         <v>100</v>
       </c>
       <c r="AS85" t="n">
-        <v>84.8</v>
+        <v>78.2</v>
       </c>
       <c r="AT85" t="inlineStr">
         <is>
@@ -17407,19 +17407,19 @@
         <v>80</v>
       </c>
       <c r="AO86" t="n">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="AP86" t="n">
         <v>30</v>
       </c>
       <c r="AQ86" t="n">
-        <v>60.8</v>
+        <v>58</v>
       </c>
       <c r="AR86" t="n">
         <v>100</v>
       </c>
       <c r="AS86" t="n">
-        <v>60.8</v>
+        <v>58</v>
       </c>
       <c r="AT86" t="inlineStr">
         <is>
@@ -17606,19 +17606,19 @@
         <v>80</v>
       </c>
       <c r="AO87" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="AP87" t="n">
         <v>30</v>
       </c>
       <c r="AQ87" t="n">
-        <v>48.4</v>
+        <v>44.8</v>
       </c>
       <c r="AR87" t="n">
         <v>100</v>
       </c>
       <c r="AS87" t="n">
-        <v>48.4</v>
+        <v>44.8</v>
       </c>
       <c r="AT87" t="inlineStr">
         <is>
@@ -17798,22 +17798,22 @@
         <v>5</v>
       </c>
       <c r="AN88" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO88" t="n">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="AP88" t="n">
         <v>30</v>
       </c>
       <c r="AQ88" t="n">
-        <v>85.2</v>
+        <v>78.2</v>
       </c>
       <c r="AR88" t="n">
         <v>100</v>
       </c>
       <c r="AS88" t="n">
-        <v>85.2</v>
+        <v>78.2</v>
       </c>
       <c r="AT88" t="inlineStr">
         <is>
@@ -17996,19 +17996,19 @@
         <v>80</v>
       </c>
       <c r="AO89" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="AP89" t="n">
         <v>30</v>
       </c>
       <c r="AQ89" t="n">
-        <v>48.4</v>
+        <v>44.8</v>
       </c>
       <c r="AR89" t="n">
         <v>100</v>
       </c>
       <c r="AS89" t="n">
-        <v>48.4</v>
+        <v>44.8</v>
       </c>
       <c r="AT89" t="inlineStr">
         <is>
@@ -18192,22 +18192,22 @@
         <v>5</v>
       </c>
       <c r="AN90" t="n">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="AO90" t="n">
-        <v>100</v>
+        <v>76</v>
       </c>
       <c r="AP90" t="n">
         <v>30</v>
       </c>
       <c r="AQ90" t="n">
-        <v>73.40000000000001</v>
+        <v>61.4</v>
       </c>
       <c r="AR90" t="n">
         <v>100</v>
       </c>
       <c r="AS90" t="n">
-        <v>73.40000000000001</v>
+        <v>61.4</v>
       </c>
       <c r="AT90" t="inlineStr">
         <is>
@@ -18391,22 +18391,22 @@
         <v>5</v>
       </c>
       <c r="AN91" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO91" t="n">
-        <v>93</v>
+        <v>62</v>
       </c>
       <c r="AP91" t="n">
         <v>30</v>
       </c>
       <c r="AQ91" t="n">
-        <v>83.2</v>
+        <v>67.8</v>
       </c>
       <c r="AR91" t="n">
         <v>100</v>
       </c>
       <c r="AS91" t="n">
-        <v>83.2</v>
+        <v>67.8</v>
       </c>
       <c r="AT91" t="inlineStr">
         <is>
@@ -18586,22 +18586,22 @@
         <v>5</v>
       </c>
       <c r="AN92" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO92" t="n">
-        <v>100</v>
+        <v>62</v>
       </c>
       <c r="AP92" t="n">
         <v>30</v>
       </c>
       <c r="AQ92" t="n">
-        <v>86</v>
+        <v>67.8</v>
       </c>
       <c r="AR92" t="n">
         <v>100</v>
       </c>
       <c r="AS92" t="n">
-        <v>86</v>
+        <v>67.8</v>
       </c>
       <c r="AT92" t="inlineStr">
         <is>
@@ -18781,22 +18781,22 @@
         <v>5</v>
       </c>
       <c r="AN93" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO93" t="n">
-        <v>98</v>
+        <v>76</v>
       </c>
       <c r="AP93" t="n">
         <v>30</v>
       </c>
       <c r="AQ93" t="n">
-        <v>85.2</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="AR93" t="n">
         <v>100</v>
       </c>
       <c r="AS93" t="n">
-        <v>85.2</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="AT93" t="inlineStr">
         <is>
@@ -18980,22 +18980,22 @@
         <v>5</v>
       </c>
       <c r="AN94" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AO94" t="n">
-        <v>53</v>
+        <v>28</v>
       </c>
       <c r="AP94" t="n">
         <v>30</v>
       </c>
       <c r="AQ94" t="n">
-        <v>67.2</v>
+        <v>51.2</v>
       </c>
       <c r="AR94" t="n">
         <v>100</v>
       </c>
       <c r="AS94" t="n">
-        <v>67.2</v>
+        <v>51.2</v>
       </c>
       <c r="AT94" t="inlineStr">
         <is>
@@ -19179,22 +19179,22 @@
         <v>5</v>
       </c>
       <c r="AN95" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AO95" t="n">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="AP95" t="n">
         <v>30</v>
       </c>
       <c r="AQ95" t="n">
-        <v>58.4</v>
+        <v>44.8</v>
       </c>
       <c r="AR95" t="n">
         <v>100</v>
       </c>
       <c r="AS95" t="n">
-        <v>58.4</v>
+        <v>44.8</v>
       </c>
       <c r="AT95" t="inlineStr">
         <is>
@@ -19377,19 +19377,19 @@
         <v>90</v>
       </c>
       <c r="AO96" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="AP96" t="n">
         <v>30</v>
       </c>
       <c r="AQ96" t="n">
-        <v>56.6</v>
+        <v>54.2</v>
       </c>
       <c r="AR96" t="n">
         <v>100</v>
       </c>
       <c r="AS96" t="n">
-        <v>56.6</v>
+        <v>54.2</v>
       </c>
       <c r="AT96" t="inlineStr">
         <is>
@@ -19573,22 +19573,22 @@
         <v>5</v>
       </c>
       <c r="AN97" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO97" t="n">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="AP97" t="n">
         <v>30</v>
       </c>
       <c r="AQ97" t="n">
-        <v>86</v>
+        <v>78.2</v>
       </c>
       <c r="AR97" t="n">
         <v>100</v>
       </c>
       <c r="AS97" t="n">
-        <v>86</v>
+        <v>78.2</v>
       </c>
       <c r="AT97" t="inlineStr">
         <is>
@@ -19779,19 +19779,19 @@
         <v>80</v>
       </c>
       <c r="AO98" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="AP98" t="n">
         <v>30</v>
       </c>
       <c r="AQ98" t="n">
-        <v>55.2</v>
+        <v>51.2</v>
       </c>
       <c r="AR98" t="n">
         <v>100</v>
       </c>
       <c r="AS98" t="n">
-        <v>55.2</v>
+        <v>51.2</v>
       </c>
       <c r="AT98" t="inlineStr">
         <is>
@@ -19975,22 +19975,22 @@
         <v>5</v>
       </c>
       <c r="AN99" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO99" t="n">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="AP99" t="n">
         <v>30</v>
       </c>
       <c r="AQ99" t="n">
-        <v>67.59999999999999</v>
+        <v>61</v>
       </c>
       <c r="AR99" t="n">
         <v>100</v>
       </c>
       <c r="AS99" t="n">
-        <v>67.59999999999999</v>
+        <v>61</v>
       </c>
       <c r="AT99" t="inlineStr">
         <is>
@@ -20177,19 +20177,19 @@
         <v>50</v>
       </c>
       <c r="AO100" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="AP100" t="n">
         <v>30</v>
       </c>
       <c r="AQ100" t="n">
-        <v>44.6</v>
+        <v>42.2</v>
       </c>
       <c r="AR100" t="n">
         <v>100</v>
       </c>
       <c r="AS100" t="n">
-        <v>44.6</v>
+        <v>42.2</v>
       </c>
       <c r="AT100" t="inlineStr">
         <is>
@@ -20376,19 +20376,19 @@
         <v>90</v>
       </c>
       <c r="AO101" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="AP101" t="n">
         <v>30</v>
       </c>
       <c r="AQ101" t="n">
-        <v>51.4</v>
+        <v>47.8</v>
       </c>
       <c r="AR101" t="n">
         <v>100</v>
       </c>
       <c r="AS101" t="n">
-        <v>51.4</v>
+        <v>47.8</v>
       </c>
       <c r="AT101" t="inlineStr">
         <is>
@@ -20575,19 +20575,19 @@
         <v>80</v>
       </c>
       <c r="AO102" t="n">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="AP102" t="n">
         <v>30</v>
       </c>
       <c r="AQ102" t="n">
-        <v>80</v>
+        <v>75.2</v>
       </c>
       <c r="AR102" t="n">
         <v>100</v>
       </c>
       <c r="AS102" t="n">
-        <v>80</v>
+        <v>75.2</v>
       </c>
       <c r="AT102" t="inlineStr">
         <is>
@@ -20767,7 +20767,7 @@
         <v>5</v>
       </c>
       <c r="AN103" t="n">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="AO103" t="n">
         <v>45</v>
@@ -20776,13 +20776,13 @@
         <v>30</v>
       </c>
       <c r="AQ103" t="n">
-        <v>60.4</v>
+        <v>58</v>
       </c>
       <c r="AR103" t="n">
         <v>100</v>
       </c>
       <c r="AS103" t="n">
-        <v>60.4</v>
+        <v>58</v>
       </c>
       <c r="AT103" t="inlineStr">
         <is>
@@ -20966,22 +20966,22 @@
         <v>5</v>
       </c>
       <c r="AN104" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="AO104" t="n">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="AP104" t="n">
         <v>30</v>
       </c>
       <c r="AQ104" t="n">
-        <v>58.5</v>
+        <v>51.2</v>
       </c>
       <c r="AR104" t="n">
         <v>100</v>
       </c>
       <c r="AS104" t="n">
-        <v>58.5</v>
+        <v>51.2</v>
       </c>
       <c r="AT104" t="inlineStr">
         <is>
@@ -21165,22 +21165,22 @@
         <v>5</v>
       </c>
       <c r="AN105" t="n">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="AO105" t="n">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="AP105" t="n">
         <v>30</v>
       </c>
       <c r="AQ105" t="n">
-        <v>76.40000000000001</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="AR105" t="n">
         <v>100</v>
       </c>
       <c r="AS105" t="n">
-        <v>76.40000000000001</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="AT105" t="inlineStr">
         <is>
@@ -21360,7 +21360,7 @@
         <v>5</v>
       </c>
       <c r="AN106" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AO106" t="n">
         <v>28</v>
@@ -21369,13 +21369,13 @@
         <v>30</v>
       </c>
       <c r="AQ106" t="n">
-        <v>56.6</v>
+        <v>54.2</v>
       </c>
       <c r="AR106" t="n">
         <v>100</v>
       </c>
       <c r="AS106" t="n">
-        <v>56.6</v>
+        <v>54.2</v>
       </c>
       <c r="AT106" t="inlineStr">
         <is>
@@ -21559,22 +21559,22 @@
         <v>5</v>
       </c>
       <c r="AN107" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AO107" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="AP107" t="n">
         <v>30</v>
       </c>
       <c r="AQ107" t="n">
-        <v>67.40000000000001</v>
+        <v>61</v>
       </c>
       <c r="AR107" t="n">
         <v>100</v>
       </c>
       <c r="AS107" t="n">
-        <v>67.40000000000001</v>
+        <v>61</v>
       </c>
       <c r="AT107" t="inlineStr">
         <is>
@@ -21758,22 +21758,22 @@
         <v>5</v>
       </c>
       <c r="AN108" t="n">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="AO108" t="n">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="AP108" t="n">
         <v>30</v>
       </c>
       <c r="AQ108" t="n">
-        <v>50.6</v>
+        <v>42.2</v>
       </c>
       <c r="AR108" t="n">
         <v>100</v>
       </c>
       <c r="AS108" t="n">
-        <v>50.6</v>
+        <v>42.2</v>
       </c>
       <c r="AT108" t="inlineStr">
         <is>
@@ -21956,19 +21956,19 @@
         <v>80</v>
       </c>
       <c r="AO109" t="n">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="AP109" t="n">
         <v>30</v>
       </c>
       <c r="AQ109" t="n">
-        <v>54.8</v>
+        <v>51.2</v>
       </c>
       <c r="AR109" t="n">
         <v>100</v>
       </c>
       <c r="AS109" t="n">
-        <v>54.8</v>
+        <v>51.2</v>
       </c>
       <c r="AT109" t="inlineStr">
         <is>
@@ -22155,19 +22155,19 @@
         <v>80</v>
       </c>
       <c r="AO110" t="n">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="AP110" t="n">
         <v>30</v>
       </c>
       <c r="AQ110" t="n">
-        <v>56.8</v>
+        <v>51.2</v>
       </c>
       <c r="AR110" t="n">
         <v>100</v>
       </c>
       <c r="AS110" t="n">
-        <v>56.8</v>
+        <v>51.2</v>
       </c>
       <c r="AT110" t="inlineStr">
         <is>
@@ -22351,22 +22351,22 @@
         <v>5</v>
       </c>
       <c r="AN111" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO111" t="n">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="AP111" t="n">
         <v>30</v>
       </c>
       <c r="AQ111" t="n">
-        <v>86</v>
+        <v>78.2</v>
       </c>
       <c r="AR111" t="n">
         <v>100</v>
       </c>
       <c r="AS111" t="n">
-        <v>86</v>
+        <v>78.2</v>
       </c>
       <c r="AT111" t="inlineStr">
         <is>
@@ -22553,19 +22553,19 @@
         <v>90</v>
       </c>
       <c r="AO112" t="n">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="AP112" t="n">
         <v>30</v>
       </c>
       <c r="AQ112" t="n">
-        <v>59.8</v>
+        <v>54.2</v>
       </c>
       <c r="AR112" t="n">
         <v>100</v>
       </c>
       <c r="AS112" t="n">
-        <v>59.8</v>
+        <v>54.2</v>
       </c>
       <c r="AT112" t="inlineStr">
         <is>
@@ -22749,22 +22749,22 @@
         <v>5</v>
       </c>
       <c r="AN113" t="n">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="AO113" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="AP113" t="n">
         <v>30</v>
       </c>
       <c r="AQ113" t="n">
-        <v>62.4</v>
+        <v>58</v>
       </c>
       <c r="AR113" t="n">
         <v>100</v>
       </c>
       <c r="AS113" t="n">
-        <v>62.4</v>
+        <v>58</v>
       </c>
       <c r="AT113" t="inlineStr">
         <is>
@@ -22951,19 +22951,19 @@
         <v>90</v>
       </c>
       <c r="AO114" t="n">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="AP114" t="n">
         <v>30</v>
       </c>
       <c r="AQ114" t="n">
-        <v>83</v>
+        <v>78.2</v>
       </c>
       <c r="AR114" t="n">
         <v>100</v>
       </c>
       <c r="AS114" t="n">
-        <v>83</v>
+        <v>78.2</v>
       </c>
       <c r="AT114" t="inlineStr">
         <is>
@@ -23151,22 +23151,22 @@
         <v>5</v>
       </c>
       <c r="AN115" t="n">
+        <v>80</v>
+      </c>
+      <c r="AO115" t="n">
         <v>88</v>
-      </c>
-      <c r="AO115" t="n">
-        <v>96</v>
       </c>
       <c r="AP115" t="n">
         <v>30</v>
       </c>
       <c r="AQ115" t="n">
-        <v>80.8</v>
+        <v>75.2</v>
       </c>
       <c r="AR115" t="n">
         <v>100</v>
       </c>
       <c r="AS115" t="n">
-        <v>80.8</v>
+        <v>75.2</v>
       </c>
       <c r="AT115" t="inlineStr">
         <is>
@@ -23354,7 +23354,7 @@
         <v>5</v>
       </c>
       <c r="AN116" t="n">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="AO116" t="n">
         <v>62</v>
@@ -23363,13 +23363,13 @@
         <v>30</v>
       </c>
       <c r="AQ116" t="n">
-        <v>60.6</v>
+        <v>55.8</v>
       </c>
       <c r="AR116" t="n">
         <v>100</v>
       </c>
       <c r="AS116" t="n">
-        <v>60.6</v>
+        <v>55.8</v>
       </c>
       <c r="AT116" t="inlineStr">
         <is>
@@ -23553,7 +23553,7 @@
         <v>5</v>
       </c>
       <c r="AN117" t="n">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="AO117" t="n">
         <v>88</v>
@@ -23562,13 +23562,13 @@
         <v>30</v>
       </c>
       <c r="AQ117" t="n">
-        <v>68.59999999999999</v>
+        <v>66.2</v>
       </c>
       <c r="AR117" t="n">
         <v>100</v>
       </c>
       <c r="AS117" t="n">
-        <v>68.59999999999999</v>
+        <v>66.2</v>
       </c>
       <c r="AT117" t="inlineStr">
         <is>
@@ -23752,22 +23752,22 @@
         <v>5</v>
       </c>
       <c r="AN118" t="n">
+        <v>80</v>
+      </c>
+      <c r="AO118" t="n">
         <v>88</v>
-      </c>
-      <c r="AO118" t="n">
-        <v>100</v>
       </c>
       <c r="AP118" t="n">
         <v>30</v>
       </c>
       <c r="AQ118" t="n">
-        <v>82.40000000000001</v>
+        <v>75.2</v>
       </c>
       <c r="AR118" t="n">
         <v>100</v>
       </c>
       <c r="AS118" t="n">
-        <v>82.40000000000001</v>
+        <v>75.2</v>
       </c>
       <c r="AT118" t="inlineStr">
         <is>
@@ -23954,19 +23954,19 @@
         <v>80</v>
       </c>
       <c r="AO119" t="n">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="AP119" t="n">
         <v>30</v>
       </c>
       <c r="AQ119" t="n">
-        <v>73.59999999999999</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="AR119" t="n">
         <v>100</v>
       </c>
       <c r="AS119" t="n">
-        <v>73.59999999999999</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="AT119" t="inlineStr">
         <is>
@@ -24153,19 +24153,19 @@
         <v>90</v>
       </c>
       <c r="AO120" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AP120" t="n">
         <v>30</v>
       </c>
       <c r="AQ120" t="n">
-        <v>47.4</v>
+        <v>47.8</v>
       </c>
       <c r="AR120" t="n">
         <v>100</v>
       </c>
       <c r="AS120" t="n">
-        <v>47.4</v>
+        <v>47.8</v>
       </c>
       <c r="AT120" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Updated CV Analysis system and deployment setup
</commit_message>
<xml_diff>
--- a/cv_analyzer/data/applicants.xlsx
+++ b/cv_analyzer/data/applicants.xlsx
@@ -832,22 +832,22 @@
         <v>5</v>
       </c>
       <c r="AN2" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AO2" t="n">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="AP2" t="n">
         <v>30</v>
       </c>
       <c r="AQ2" t="n">
-        <v>73.40000000000001</v>
+        <v>67.8</v>
       </c>
       <c r="AR2" t="n">
         <v>100</v>
       </c>
       <c r="AS2" t="n">
-        <v>73.40000000000001</v>
+        <v>67.8</v>
       </c>
       <c r="AT2" t="inlineStr">
         <is>
@@ -996,25 +996,25 @@
         <v>5</v>
       </c>
       <c r="AM3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AN3" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="AO3" t="n">
         <v>12</v>
       </c>
       <c r="AP3" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="AQ3" t="n">
-        <v>16.3</v>
+        <v>32.8</v>
       </c>
       <c r="AR3" t="n">
         <v>100</v>
       </c>
       <c r="AS3" t="n">
-        <v>16.3</v>
+        <v>32.8</v>
       </c>
       <c r="AT3" t="inlineStr">
         <is>
@@ -1193,19 +1193,19 @@
         <v>80</v>
       </c>
       <c r="AO4" t="n">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="AP4" t="n">
         <v>30</v>
       </c>
       <c r="AQ4" t="n">
-        <v>56</v>
+        <v>44.8</v>
       </c>
       <c r="AR4" t="n">
         <v>100</v>
       </c>
       <c r="AS4" t="n">
-        <v>56</v>
+        <v>44.8</v>
       </c>
       <c r="AT4" t="inlineStr">
         <is>
@@ -1392,19 +1392,19 @@
         <v>80</v>
       </c>
       <c r="AO5" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="AP5" t="n">
         <v>30</v>
       </c>
       <c r="AQ5" t="n">
-        <v>63.6</v>
+        <v>58</v>
       </c>
       <c r="AR5" t="n">
         <v>100</v>
       </c>
       <c r="AS5" t="n">
-        <v>63.6</v>
+        <v>58</v>
       </c>
       <c r="AT5" t="inlineStr">
         <is>
@@ -1779,22 +1779,22 @@
         <v>5</v>
       </c>
       <c r="AN7" t="n">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="AO7" t="n">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="AP7" t="n">
         <v>30</v>
       </c>
       <c r="AQ7" t="n">
-        <v>75.8</v>
+        <v>66.2</v>
       </c>
       <c r="AR7" t="n">
         <v>100</v>
       </c>
       <c r="AS7" t="n">
-        <v>75.8</v>
+        <v>66.2</v>
       </c>
       <c r="AT7" t="inlineStr">
         <is>
@@ -1978,22 +1978,22 @@
         <v>5</v>
       </c>
       <c r="AN8" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AO8" t="n">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="AP8" t="n">
         <v>30</v>
       </c>
       <c r="AQ8" t="n">
-        <v>74.2</v>
+        <v>67.8</v>
       </c>
       <c r="AR8" t="n">
         <v>100</v>
       </c>
       <c r="AS8" t="n">
-        <v>74.2</v>
+        <v>67.8</v>
       </c>
       <c r="AT8" t="inlineStr">
         <is>
@@ -2176,19 +2176,19 @@
         <v>50</v>
       </c>
       <c r="AO9" t="n">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="AP9" t="n">
         <v>30</v>
       </c>
       <c r="AQ9" t="n">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="AR9" t="n">
         <v>100</v>
       </c>
       <c r="AS9" t="n">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="AT9" t="inlineStr">
         <is>
@@ -2368,22 +2368,22 @@
         <v>5</v>
       </c>
       <c r="AN10" t="n">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="AO10" t="n">
-        <v>65</v>
+        <v>45</v>
       </c>
       <c r="AP10" t="n">
         <v>30</v>
       </c>
       <c r="AQ10" t="n">
-        <v>70.8</v>
+        <v>58</v>
       </c>
       <c r="AR10" t="n">
         <v>100</v>
       </c>
       <c r="AS10" t="n">
-        <v>70.8</v>
+        <v>58</v>
       </c>
       <c r="AT10" t="inlineStr">
         <is>
@@ -2570,19 +2570,19 @@
         <v>90</v>
       </c>
       <c r="AO11" t="n">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="AP11" t="n">
         <v>30</v>
       </c>
       <c r="AQ11" t="n">
-        <v>57</v>
+        <v>54.2</v>
       </c>
       <c r="AR11" t="n">
         <v>100</v>
       </c>
       <c r="AS11" t="n">
-        <v>57</v>
+        <v>54.2</v>
       </c>
       <c r="AT11" t="inlineStr">
         <is>
@@ -2766,22 +2766,22 @@
         <v>5</v>
       </c>
       <c r="AN12" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AO12" t="n">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="AP12" t="n">
         <v>30</v>
       </c>
       <c r="AQ12" t="n">
-        <v>67.59999999999999</v>
+        <v>58</v>
       </c>
       <c r="AR12" t="n">
         <v>100</v>
       </c>
       <c r="AS12" t="n">
-        <v>67.59999999999999</v>
+        <v>58</v>
       </c>
       <c r="AT12" t="inlineStr">
         <is>
@@ -2965,7 +2965,7 @@
         <v>5</v>
       </c>
       <c r="AN13" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO13" t="n">
         <v>12</v>
@@ -2974,13 +2974,13 @@
         <v>30</v>
       </c>
       <c r="AQ13" t="n">
-        <v>50.8</v>
+        <v>47.8</v>
       </c>
       <c r="AR13" t="n">
         <v>100</v>
       </c>
       <c r="AS13" t="n">
-        <v>50.8</v>
+        <v>47.8</v>
       </c>
       <c r="AT13" t="inlineStr">
         <is>
@@ -3164,22 +3164,22 @@
         <v>5</v>
       </c>
       <c r="AN14" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AO14" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="AP14" t="n">
         <v>30</v>
       </c>
       <c r="AQ14" t="n">
-        <v>83.8</v>
+        <v>78.2</v>
       </c>
       <c r="AR14" t="n">
         <v>100</v>
       </c>
       <c r="AS14" t="n">
-        <v>83.8</v>
+        <v>78.2</v>
       </c>
       <c r="AT14" t="inlineStr">
         <is>
@@ -3359,22 +3359,22 @@
         <v>5</v>
       </c>
       <c r="AN15" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AO15" t="n">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="AP15" t="n">
         <v>30</v>
       </c>
       <c r="AQ15" t="n">
-        <v>60.2</v>
+        <v>54.2</v>
       </c>
       <c r="AR15" t="n">
         <v>100</v>
       </c>
       <c r="AS15" t="n">
-        <v>60.2</v>
+        <v>54.2</v>
       </c>
       <c r="AT15" t="inlineStr">
         <is>
@@ -3565,19 +3565,19 @@
         <v>90</v>
       </c>
       <c r="AO16" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="AP16" t="n">
         <v>30</v>
       </c>
       <c r="AQ16" t="n">
-        <v>67.40000000000001</v>
+        <v>67.8</v>
       </c>
       <c r="AR16" t="n">
         <v>100</v>
       </c>
       <c r="AS16" t="n">
-        <v>67.40000000000001</v>
+        <v>67.8</v>
       </c>
       <c r="AT16" t="inlineStr">
         <is>
@@ -3761,22 +3761,22 @@
         <v>5</v>
       </c>
       <c r="AN17" t="n">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="AO17" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="AP17" t="n">
         <v>30</v>
       </c>
       <c r="AQ17" t="n">
-        <v>42.2</v>
+        <v>35.8</v>
       </c>
       <c r="AR17" t="n">
         <v>100</v>
       </c>
       <c r="AS17" t="n">
-        <v>42.2</v>
+        <v>35.8</v>
       </c>
       <c r="AT17" t="inlineStr">
         <is>
@@ -3960,7 +3960,7 @@
         <v>5</v>
       </c>
       <c r="AN18" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AO18" t="n">
         <v>28</v>
@@ -3969,13 +3969,13 @@
         <v>30</v>
       </c>
       <c r="AQ18" t="n">
-        <v>57.2</v>
+        <v>51.2</v>
       </c>
       <c r="AR18" t="n">
         <v>100</v>
       </c>
       <c r="AS18" t="n">
-        <v>57.2</v>
+        <v>51.2</v>
       </c>
       <c r="AT18" t="inlineStr">
         <is>
@@ -4152,25 +4152,25 @@
         <v>5</v>
       </c>
       <c r="AM19" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AN19" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AO19" t="n">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="AP19" t="n">
         <v>30</v>
       </c>
       <c r="AQ19" t="n">
-        <v>80.40000000000001</v>
+        <v>78.2</v>
       </c>
       <c r="AR19" t="n">
         <v>100</v>
       </c>
       <c r="AS19" t="n">
-        <v>80.40000000000001</v>
+        <v>78.2</v>
       </c>
       <c r="AT19" t="inlineStr">
         <is>
@@ -4354,22 +4354,22 @@
         <v>5</v>
       </c>
       <c r="AN20" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AO20" t="n">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="AP20" t="n">
         <v>30</v>
       </c>
       <c r="AQ20" t="n">
-        <v>85.40000000000001</v>
+        <v>78.2</v>
       </c>
       <c r="AR20" t="n">
         <v>100</v>
       </c>
       <c r="AS20" t="n">
-        <v>85.40000000000001</v>
+        <v>78.2</v>
       </c>
       <c r="AT20" t="inlineStr">
         <is>
@@ -4553,22 +4553,22 @@
         <v>5</v>
       </c>
       <c r="AN21" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AO21" t="n">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="AP21" t="n">
         <v>30</v>
       </c>
       <c r="AQ21" t="n">
-        <v>57.8</v>
+        <v>47.8</v>
       </c>
       <c r="AR21" t="n">
         <v>100</v>
       </c>
       <c r="AS21" t="n">
-        <v>57.8</v>
+        <v>47.8</v>
       </c>
       <c r="AT21" t="inlineStr">
         <is>
@@ -4752,22 +4752,22 @@
         <v>5</v>
       </c>
       <c r="AN22" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO22" t="n">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="AP22" t="n">
         <v>30</v>
       </c>
       <c r="AQ22" t="n">
-        <v>56.8</v>
+        <v>47.8</v>
       </c>
       <c r="AR22" t="n">
         <v>100</v>
       </c>
       <c r="AS22" t="n">
-        <v>56.8</v>
+        <v>47.8</v>
       </c>
       <c r="AT22" t="inlineStr">
         <is>
@@ -4951,22 +4951,22 @@
         <v>5</v>
       </c>
       <c r="AN23" t="n">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="AO23" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="AP23" t="n">
         <v>30</v>
       </c>
       <c r="AQ23" t="n">
-        <v>43</v>
+        <v>35.8</v>
       </c>
       <c r="AR23" t="n">
         <v>100</v>
       </c>
       <c r="AS23" t="n">
-        <v>43</v>
+        <v>35.8</v>
       </c>
       <c r="AT23" t="inlineStr">
         <is>
@@ -5150,7 +5150,7 @@
         <v>5</v>
       </c>
       <c r="AN24" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO24" t="n">
         <v>28</v>
@@ -5159,13 +5159,13 @@
         <v>30</v>
       </c>
       <c r="AQ24" t="n">
-        <v>57.2</v>
+        <v>54.2</v>
       </c>
       <c r="AR24" t="n">
         <v>100</v>
       </c>
       <c r="AS24" t="n">
-        <v>57.2</v>
+        <v>54.2</v>
       </c>
       <c r="AT24" t="inlineStr">
         <is>
@@ -5349,22 +5349,22 @@
         <v>5</v>
       </c>
       <c r="AN25" t="n">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="AO25" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="AP25" t="n">
         <v>30</v>
       </c>
       <c r="AQ25" t="n">
-        <v>77.59999999999999</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="AR25" t="n">
         <v>100</v>
       </c>
       <c r="AS25" t="n">
-        <v>77.59999999999999</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="AT25" t="inlineStr">
         <is>
@@ -5548,22 +5548,22 @@
         <v>5</v>
       </c>
       <c r="AN26" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO26" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="AP26" t="n">
         <v>30</v>
       </c>
       <c r="AQ26" t="n">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="AR26" t="n">
         <v>100</v>
       </c>
       <c r="AS26" t="n">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="AT26" t="inlineStr">
         <is>
@@ -5743,22 +5743,22 @@
         <v>5</v>
       </c>
       <c r="AN27" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AO27" t="n">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="AP27" t="n">
         <v>30</v>
       </c>
       <c r="AQ27" t="n">
-        <v>74.2</v>
+        <v>67.8</v>
       </c>
       <c r="AR27" t="n">
         <v>100</v>
       </c>
       <c r="AS27" t="n">
-        <v>74.2</v>
+        <v>67.8</v>
       </c>
       <c r="AT27" t="inlineStr">
         <is>
@@ -5938,22 +5938,22 @@
         <v>5</v>
       </c>
       <c r="AN28" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO28" t="n">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="AP28" t="n">
         <v>30</v>
       </c>
       <c r="AQ28" t="n">
-        <v>86</v>
+        <v>78.2</v>
       </c>
       <c r="AR28" t="n">
         <v>100</v>
       </c>
       <c r="AS28" t="n">
-        <v>86</v>
+        <v>78.2</v>
       </c>
       <c r="AT28" t="inlineStr">
         <is>
@@ -6137,7 +6137,7 @@
         <v>5</v>
       </c>
       <c r="AN29" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AO29" t="n">
         <v>28</v>
@@ -6146,13 +6146,13 @@
         <v>30</v>
       </c>
       <c r="AQ29" t="n">
-        <v>57.2</v>
+        <v>51.2</v>
       </c>
       <c r="AR29" t="n">
         <v>100</v>
       </c>
       <c r="AS29" t="n">
-        <v>57.2</v>
+        <v>51.2</v>
       </c>
       <c r="AT29" t="inlineStr">
         <is>
@@ -6336,22 +6336,22 @@
         <v>5</v>
       </c>
       <c r="AN30" t="n">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="AO30" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="AP30" t="n">
         <v>30</v>
       </c>
       <c r="AQ30" t="n">
-        <v>72</v>
+        <v>64.8</v>
       </c>
       <c r="AR30" t="n">
         <v>100</v>
       </c>
       <c r="AS30" t="n">
-        <v>72</v>
+        <v>64.8</v>
       </c>
       <c r="AT30" t="inlineStr">
         <is>
@@ -6535,22 +6535,22 @@
         <v>5</v>
       </c>
       <c r="AN31" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="AO31" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="AP31" t="n">
         <v>30</v>
       </c>
       <c r="AQ31" t="n">
-        <v>29.3</v>
+        <v>35.8</v>
       </c>
       <c r="AR31" t="n">
         <v>100</v>
       </c>
       <c r="AS31" t="n">
-        <v>29.3</v>
+        <v>35.8</v>
       </c>
       <c r="AT31" t="inlineStr">
         <is>
@@ -6730,22 +6730,22 @@
         <v>5</v>
       </c>
       <c r="AN32" t="n">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="AO32" t="n">
-        <v>99</v>
+        <v>62</v>
       </c>
       <c r="AP32" t="n">
         <v>30</v>
       </c>
       <c r="AQ32" t="n">
-        <v>84.40000000000001</v>
+        <v>64.8</v>
       </c>
       <c r="AR32" t="n">
         <v>100</v>
       </c>
       <c r="AS32" t="n">
-        <v>84.40000000000001</v>
+        <v>64.8</v>
       </c>
       <c r="AT32" t="inlineStr">
         <is>
@@ -6929,7 +6929,7 @@
         <v>5</v>
       </c>
       <c r="AN33" t="n">
-        <v>74</v>
+        <v>50</v>
       </c>
       <c r="AO33" t="n">
         <v>12</v>
@@ -6938,13 +6938,13 @@
         <v>30</v>
       </c>
       <c r="AQ33" t="n">
-        <v>43</v>
+        <v>35.8</v>
       </c>
       <c r="AR33" t="n">
         <v>100</v>
       </c>
       <c r="AS33" t="n">
-        <v>43</v>
+        <v>35.8</v>
       </c>
       <c r="AT33" t="inlineStr">
         <is>
@@ -7128,22 +7128,22 @@
         <v>5</v>
       </c>
       <c r="AN34" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AO34" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="AP34" t="n">
         <v>30</v>
       </c>
       <c r="AQ34" t="n">
-        <v>53.8</v>
+        <v>47.8</v>
       </c>
       <c r="AR34" t="n">
         <v>100</v>
       </c>
       <c r="AS34" t="n">
-        <v>53.8</v>
+        <v>47.8</v>
       </c>
       <c r="AT34" t="inlineStr">
         <is>
@@ -7330,19 +7330,19 @@
         <v>80</v>
       </c>
       <c r="AO35" t="n">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="AP35" t="n">
         <v>30</v>
       </c>
       <c r="AQ35" t="n">
-        <v>55.6</v>
+        <v>51.2</v>
       </c>
       <c r="AR35" t="n">
         <v>100</v>
       </c>
       <c r="AS35" t="n">
-        <v>55.6</v>
+        <v>51.2</v>
       </c>
       <c r="AT35" t="inlineStr">
         <is>
@@ -7526,22 +7526,22 @@
         <v>5</v>
       </c>
       <c r="AN36" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AO36" t="n">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="AP36" t="n">
         <v>30</v>
       </c>
       <c r="AQ36" t="n">
-        <v>65.40000000000001</v>
+        <v>54.2</v>
       </c>
       <c r="AR36" t="n">
         <v>100</v>
       </c>
       <c r="AS36" t="n">
-        <v>65.40000000000001</v>
+        <v>54.2</v>
       </c>
       <c r="AT36" t="inlineStr">
         <is>
@@ -7732,19 +7732,19 @@
         <v>50</v>
       </c>
       <c r="AO37" t="n">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="AP37" t="n">
         <v>30</v>
       </c>
       <c r="AQ37" t="n">
-        <v>68.2</v>
+        <v>66.2</v>
       </c>
       <c r="AR37" t="n">
         <v>100</v>
       </c>
       <c r="AS37" t="n">
-        <v>68.2</v>
+        <v>66.2</v>
       </c>
       <c r="AT37" t="inlineStr">
         <is>
@@ -8130,19 +8130,19 @@
         <v>80</v>
       </c>
       <c r="AO39" t="n">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="AP39" t="n">
         <v>30</v>
       </c>
       <c r="AQ39" t="n">
-        <v>57.2</v>
+        <v>51.2</v>
       </c>
       <c r="AR39" t="n">
         <v>100</v>
       </c>
       <c r="AS39" t="n">
-        <v>57.2</v>
+        <v>51.2</v>
       </c>
       <c r="AT39" t="inlineStr">
         <is>
@@ -8317,19 +8317,19 @@
         <v>90</v>
       </c>
       <c r="AO40" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="AP40" t="n">
         <v>30</v>
       </c>
       <c r="AQ40" t="n">
-        <v>51.4</v>
+        <v>47.8</v>
       </c>
       <c r="AR40" t="n">
         <v>100</v>
       </c>
       <c r="AS40" t="n">
-        <v>51.4</v>
+        <v>47.8</v>
       </c>
       <c r="AT40" t="inlineStr">
         <is>
@@ -8512,19 +8512,19 @@
         <v>80</v>
       </c>
       <c r="AO41" t="n">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="AP41" t="n">
         <v>30</v>
       </c>
       <c r="AQ41" t="n">
-        <v>80</v>
+        <v>75.2</v>
       </c>
       <c r="AR41" t="n">
         <v>100</v>
       </c>
       <c r="AS41" t="n">
-        <v>80</v>
+        <v>75.2</v>
       </c>
       <c r="AT41" t="inlineStr">
         <is>
@@ -8685,7 +8685,7 @@
         <v>5</v>
       </c>
       <c r="AM42" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AN42" t="n">
         <v>80</v>
@@ -8697,13 +8697,13 @@
         <v>30</v>
       </c>
       <c r="AQ42" t="n">
-        <v>41.8</v>
+        <v>44.8</v>
       </c>
       <c r="AR42" t="n">
         <v>100</v>
       </c>
       <c r="AS42" t="n">
-        <v>41.8</v>
+        <v>44.8</v>
       </c>
       <c r="AT42" t="inlineStr">
         <is>
@@ -8887,7 +8887,7 @@
         <v>5</v>
       </c>
       <c r="AN43" t="n">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="AO43" t="n">
         <v>88</v>
@@ -8896,13 +8896,13 @@
         <v>30</v>
       </c>
       <c r="AQ43" t="n">
-        <v>68.59999999999999</v>
+        <v>66.2</v>
       </c>
       <c r="AR43" t="n">
         <v>100</v>
       </c>
       <c r="AS43" t="n">
-        <v>68.59999999999999</v>
+        <v>66.2</v>
       </c>
       <c r="AT43" t="inlineStr">
         <is>
@@ -9070,22 +9070,22 @@
         <v>5</v>
       </c>
       <c r="AN44" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="AO44" t="n">
         <v>12</v>
       </c>
       <c r="AP44" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="AQ44" t="n">
-        <v>22.3</v>
+        <v>34.2</v>
       </c>
       <c r="AR44" t="n">
         <v>100</v>
       </c>
       <c r="AS44" t="n">
-        <v>22.3</v>
+        <v>34.2</v>
       </c>
       <c r="AT44" t="inlineStr">
         <is>
@@ -9269,22 +9269,22 @@
         <v>5</v>
       </c>
       <c r="AN45" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AO45" t="n">
-        <v>78</v>
+        <v>45</v>
       </c>
       <c r="AP45" t="n">
         <v>30</v>
       </c>
       <c r="AQ45" t="n">
-        <v>76.59999999999999</v>
+        <v>61</v>
       </c>
       <c r="AR45" t="n">
         <v>100</v>
       </c>
       <c r="AS45" t="n">
-        <v>76.59999999999999</v>
+        <v>61</v>
       </c>
       <c r="AT45" t="inlineStr">
         <is>
@@ -9667,22 +9667,22 @@
         <v>5</v>
       </c>
       <c r="AN47" t="n">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="AO47" t="n">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="AP47" t="n">
         <v>30</v>
       </c>
       <c r="AQ47" t="n">
-        <v>60.4</v>
+        <v>51.2</v>
       </c>
       <c r="AR47" t="n">
         <v>100</v>
       </c>
       <c r="AS47" t="n">
-        <v>60.4</v>
+        <v>51.2</v>
       </c>
       <c r="AT47" t="inlineStr">
         <is>
@@ -10064,19 +10064,19 @@
         <v>90</v>
       </c>
       <c r="AO49" t="n">
-        <v>65</v>
+        <v>28</v>
       </c>
       <c r="AP49" t="n">
         <v>30</v>
       </c>
       <c r="AQ49" t="n">
-        <v>69</v>
+        <v>54.2</v>
       </c>
       <c r="AR49" t="n">
         <v>100</v>
       </c>
       <c r="AS49" t="n">
-        <v>69</v>
+        <v>54.2</v>
       </c>
       <c r="AT49" t="inlineStr">
         <is>
@@ -10264,7 +10264,7 @@
         <v>5</v>
       </c>
       <c r="AN50" t="n">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="AO50" t="n">
         <v>12</v>
@@ -10273,13 +10273,13 @@
         <v>30</v>
       </c>
       <c r="AQ50" t="n">
-        <v>47.2</v>
+        <v>44.8</v>
       </c>
       <c r="AR50" t="n">
         <v>100</v>
       </c>
       <c r="AS50" t="n">
-        <v>47.2</v>
+        <v>44.8</v>
       </c>
       <c r="AT50" t="inlineStr">
         <is>
@@ -10463,22 +10463,22 @@
         <v>5</v>
       </c>
       <c r="AN51" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AO51" t="n">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="AP51" t="n">
         <v>30</v>
       </c>
       <c r="AQ51" t="n">
-        <v>83.40000000000001</v>
+        <v>78.2</v>
       </c>
       <c r="AR51" t="n">
         <v>100</v>
       </c>
       <c r="AS51" t="n">
-        <v>83.40000000000001</v>
+        <v>78.2</v>
       </c>
       <c r="AT51" t="inlineStr">
         <is>
@@ -10861,22 +10861,22 @@
         <v>5</v>
       </c>
       <c r="AN53" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AO53" t="n">
-        <v>85</v>
+        <v>45</v>
       </c>
       <c r="AP53" t="n">
         <v>30</v>
       </c>
       <c r="AQ53" t="n">
-        <v>79.40000000000001</v>
+        <v>61</v>
       </c>
       <c r="AR53" t="n">
         <v>100</v>
       </c>
       <c r="AS53" t="n">
-        <v>79.40000000000001</v>
+        <v>61</v>
       </c>
       <c r="AT53" t="inlineStr">
         <is>
@@ -11059,19 +11059,19 @@
         <v>90</v>
       </c>
       <c r="AO54" t="n">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="AP54" t="n">
         <v>30</v>
       </c>
       <c r="AQ54" t="n">
-        <v>67</v>
+        <v>54.2</v>
       </c>
       <c r="AR54" t="n">
         <v>100</v>
       </c>
       <c r="AS54" t="n">
-        <v>67</v>
+        <v>54.2</v>
       </c>
       <c r="AT54" t="inlineStr">
         <is>
@@ -11255,22 +11255,22 @@
         <v>5</v>
       </c>
       <c r="AN55" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AO55" t="n">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="AP55" t="n">
         <v>30</v>
       </c>
       <c r="AQ55" t="n">
-        <v>85.40000000000001</v>
+        <v>78.2</v>
       </c>
       <c r="AR55" t="n">
         <v>100</v>
       </c>
       <c r="AS55" t="n">
-        <v>85.40000000000001</v>
+        <v>78.2</v>
       </c>
       <c r="AT55" t="inlineStr">
         <is>
@@ -11454,22 +11454,22 @@
         <v>5</v>
       </c>
       <c r="AN56" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO56" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="AP56" t="n">
         <v>30</v>
       </c>
       <c r="AQ56" t="n">
-        <v>66.8</v>
+        <v>54.2</v>
       </c>
       <c r="AR56" t="n">
         <v>100</v>
       </c>
       <c r="AS56" t="n">
-        <v>66.8</v>
+        <v>54.2</v>
       </c>
       <c r="AT56" t="inlineStr">
         <is>
@@ -11656,19 +11656,19 @@
         <v>90</v>
       </c>
       <c r="AO57" t="n">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="AP57" t="n">
         <v>30</v>
       </c>
       <c r="AQ57" t="n">
-        <v>60.2</v>
+        <v>47.8</v>
       </c>
       <c r="AR57" t="n">
         <v>100</v>
       </c>
       <c r="AS57" t="n">
-        <v>60.2</v>
+        <v>47.8</v>
       </c>
       <c r="AT57" t="inlineStr">
         <is>
@@ -11859,19 +11859,19 @@
         <v>90</v>
       </c>
       <c r="AO58" t="n">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="AP58" t="n">
         <v>30</v>
       </c>
       <c r="AQ58" t="n">
-        <v>81.8</v>
+        <v>78.2</v>
       </c>
       <c r="AR58" t="n">
         <v>100</v>
       </c>
       <c r="AS58" t="n">
-        <v>81.8</v>
+        <v>78.2</v>
       </c>
       <c r="AT58" t="inlineStr">
         <is>
@@ -12054,19 +12054,19 @@
         <v>90</v>
       </c>
       <c r="AO59" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="AP59" t="n">
         <v>30</v>
       </c>
       <c r="AQ59" t="n">
-        <v>56.2</v>
+        <v>54.2</v>
       </c>
       <c r="AR59" t="n">
         <v>100</v>
       </c>
       <c r="AS59" t="n">
-        <v>56.2</v>
+        <v>54.2</v>
       </c>
       <c r="AT59" t="inlineStr">
         <is>
@@ -12253,19 +12253,19 @@
         <v>90</v>
       </c>
       <c r="AO60" t="n">
-        <v>78</v>
+        <v>45</v>
       </c>
       <c r="AP60" t="n">
         <v>30</v>
       </c>
       <c r="AQ60" t="n">
-        <v>74.2</v>
+        <v>61</v>
       </c>
       <c r="AR60" t="n">
         <v>100</v>
       </c>
       <c r="AS60" t="n">
-        <v>74.2</v>
+        <v>61</v>
       </c>
       <c r="AT60" t="inlineStr">
         <is>
@@ -12449,7 +12449,7 @@
         <v>5</v>
       </c>
       <c r="AN61" t="n">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="AO61" t="n">
         <v>76</v>
@@ -12458,13 +12458,13 @@
         <v>30</v>
       </c>
       <c r="AQ61" t="n">
-        <v>72.8</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="AR61" t="n">
         <v>100</v>
       </c>
       <c r="AS61" t="n">
-        <v>72.8</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="AT61" t="inlineStr">
         <is>
@@ -12640,22 +12640,22 @@
         <v>5</v>
       </c>
       <c r="AN62" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AO62" t="n">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="AP62" t="n">
         <v>30</v>
       </c>
       <c r="AQ62" t="n">
-        <v>60.2</v>
+        <v>54.2</v>
       </c>
       <c r="AR62" t="n">
         <v>100</v>
       </c>
       <c r="AS62" t="n">
-        <v>60.2</v>
+        <v>54.2</v>
       </c>
       <c r="AT62" t="inlineStr">
         <is>
@@ -12839,22 +12839,22 @@
         <v>5</v>
       </c>
       <c r="AN63" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AO63" t="n">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="AP63" t="n">
         <v>30</v>
       </c>
       <c r="AQ63" t="n">
-        <v>74.40000000000001</v>
+        <v>64.8</v>
       </c>
       <c r="AR63" t="n">
         <v>100</v>
       </c>
       <c r="AS63" t="n">
-        <v>74.40000000000001</v>
+        <v>64.8</v>
       </c>
       <c r="AT63" t="inlineStr">
         <is>
@@ -13038,22 +13038,22 @@
         <v>5</v>
       </c>
       <c r="AN64" t="n">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="AO64" t="n">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="AP64" t="n">
         <v>30</v>
       </c>
       <c r="AQ64" t="n">
-        <v>58.4</v>
+        <v>51.2</v>
       </c>
       <c r="AR64" t="n">
         <v>100</v>
       </c>
       <c r="AS64" t="n">
-        <v>58.4</v>
+        <v>51.2</v>
       </c>
       <c r="AT64" t="inlineStr">
         <is>
@@ -13237,22 +13237,22 @@
         <v>5</v>
       </c>
       <c r="AN65" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AO65" t="n">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="AP65" t="n">
         <v>30</v>
       </c>
       <c r="AQ65" t="n">
-        <v>85.40000000000001</v>
+        <v>78.2</v>
       </c>
       <c r="AR65" t="n">
         <v>100</v>
       </c>
       <c r="AS65" t="n">
-        <v>85.40000000000001</v>
+        <v>78.2</v>
       </c>
       <c r="AT65" t="inlineStr">
         <is>
@@ -13439,19 +13439,19 @@
         <v>90</v>
       </c>
       <c r="AO66" t="n">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="AP66" t="n">
         <v>30</v>
       </c>
       <c r="AQ66" t="n">
-        <v>83</v>
+        <v>78.2</v>
       </c>
       <c r="AR66" t="n">
         <v>100</v>
       </c>
       <c r="AS66" t="n">
-        <v>83</v>
+        <v>78.2</v>
       </c>
       <c r="AT66" t="inlineStr">
         <is>
@@ -13638,19 +13638,19 @@
         <v>80</v>
       </c>
       <c r="AO67" t="n">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="AP67" t="n">
         <v>30</v>
       </c>
       <c r="AQ67" t="n">
-        <v>58.4</v>
+        <v>51.2</v>
       </c>
       <c r="AR67" t="n">
         <v>100</v>
       </c>
       <c r="AS67" t="n">
-        <v>58.4</v>
+        <v>51.2</v>
       </c>
       <c r="AT67" t="inlineStr">
         <is>
@@ -14036,19 +14036,19 @@
         <v>50</v>
       </c>
       <c r="AO69" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="AP69" t="n">
         <v>30</v>
       </c>
       <c r="AQ69" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="AR69" t="n">
         <v>100</v>
       </c>
       <c r="AS69" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="AT69" t="inlineStr">
         <is>
@@ -14232,22 +14232,22 @@
         <v>5</v>
       </c>
       <c r="AN70" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO70" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="AP70" t="n">
         <v>30</v>
       </c>
       <c r="AQ70" t="n">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="AR70" t="n">
         <v>100</v>
       </c>
       <c r="AS70" t="n">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="AT70" t="inlineStr">
         <is>
@@ -14427,22 +14427,22 @@
         <v>5</v>
       </c>
       <c r="AN71" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO71" t="n">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="AP71" t="n">
         <v>30</v>
       </c>
       <c r="AQ71" t="n">
-        <v>67.2</v>
+        <v>61</v>
       </c>
       <c r="AR71" t="n">
         <v>100</v>
       </c>
       <c r="AS71" t="n">
-        <v>67.2</v>
+        <v>61</v>
       </c>
       <c r="AT71" t="inlineStr">
         <is>
@@ -14618,22 +14618,22 @@
         <v>5</v>
       </c>
       <c r="AN72" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AO72" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="AP72" t="n">
         <v>30</v>
       </c>
       <c r="AQ72" t="n">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="AR72" t="n">
         <v>100</v>
       </c>
       <c r="AS72" t="n">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="AT72" t="inlineStr">
         <is>
@@ -14816,19 +14816,19 @@
         <v>90</v>
       </c>
       <c r="AO73" t="n">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="AP73" t="n">
         <v>30</v>
       </c>
       <c r="AQ73" t="n">
-        <v>60.2</v>
+        <v>54.2</v>
       </c>
       <c r="AR73" t="n">
         <v>100</v>
       </c>
       <c r="AS73" t="n">
-        <v>60.2</v>
+        <v>54.2</v>
       </c>
       <c r="AT73" t="inlineStr">
         <is>
@@ -15207,22 +15207,22 @@
         <v>5</v>
       </c>
       <c r="AN75" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AO75" t="n">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="AP75" t="n">
         <v>30</v>
       </c>
       <c r="AQ75" t="n">
-        <v>64.59999999999999</v>
+        <v>54.2</v>
       </c>
       <c r="AR75" t="n">
         <v>100</v>
       </c>
       <c r="AS75" t="n">
-        <v>64.59999999999999</v>
+        <v>54.2</v>
       </c>
       <c r="AT75" t="inlineStr">
         <is>
@@ -15406,22 +15406,22 @@
         <v>5</v>
       </c>
       <c r="AN76" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO76" t="n">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="AP76" t="n">
         <v>30</v>
       </c>
       <c r="AQ76" t="n">
-        <v>84.8</v>
+        <v>78.2</v>
       </c>
       <c r="AR76" t="n">
         <v>100</v>
       </c>
       <c r="AS76" t="n">
-        <v>84.8</v>
+        <v>78.2</v>
       </c>
       <c r="AT76" t="inlineStr">
         <is>
@@ -15605,22 +15605,22 @@
         <v>5</v>
       </c>
       <c r="AN77" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO77" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="AP77" t="n">
         <v>30</v>
       </c>
       <c r="AQ77" t="n">
-        <v>54</v>
+        <v>47.8</v>
       </c>
       <c r="AR77" t="n">
         <v>100</v>
       </c>
       <c r="AS77" t="n">
-        <v>54</v>
+        <v>47.8</v>
       </c>
       <c r="AT77" t="inlineStr">
         <is>
@@ -15804,7 +15804,7 @@
         <v>5</v>
       </c>
       <c r="AN78" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AO78" t="n">
         <v>28</v>
@@ -15813,13 +15813,13 @@
         <v>30</v>
       </c>
       <c r="AQ78" t="n">
-        <v>56.6</v>
+        <v>54.2</v>
       </c>
       <c r="AR78" t="n">
         <v>100</v>
       </c>
       <c r="AS78" t="n">
-        <v>56.6</v>
+        <v>54.2</v>
       </c>
       <c r="AT78" t="inlineStr">
         <is>
@@ -16003,22 +16003,22 @@
         <v>5</v>
       </c>
       <c r="AN79" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AO79" t="n">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="AP79" t="n">
         <v>30</v>
       </c>
       <c r="AQ79" t="n">
-        <v>67.59999999999999</v>
+        <v>58</v>
       </c>
       <c r="AR79" t="n">
         <v>100</v>
       </c>
       <c r="AS79" t="n">
-        <v>67.59999999999999</v>
+        <v>58</v>
       </c>
       <c r="AT79" t="inlineStr">
         <is>
@@ -16206,22 +16206,22 @@
         <v>5</v>
       </c>
       <c r="AN80" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO80" t="n">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="AP80" t="n">
         <v>30</v>
       </c>
       <c r="AQ80" t="n">
-        <v>85.2</v>
+        <v>78.2</v>
       </c>
       <c r="AR80" t="n">
         <v>100</v>
       </c>
       <c r="AS80" t="n">
-        <v>85.2</v>
+        <v>78.2</v>
       </c>
       <c r="AT80" t="inlineStr">
         <is>
@@ -16409,22 +16409,22 @@
         <v>5</v>
       </c>
       <c r="AN81" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO81" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="AP81" t="n">
         <v>30</v>
       </c>
       <c r="AQ81" t="n">
-        <v>69.59999999999999</v>
+        <v>61</v>
       </c>
       <c r="AR81" t="n">
         <v>100</v>
       </c>
       <c r="AS81" t="n">
-        <v>69.59999999999999</v>
+        <v>61</v>
       </c>
       <c r="AT81" t="inlineStr">
         <is>
@@ -16608,22 +16608,22 @@
         <v>5</v>
       </c>
       <c r="AN82" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AO82" t="n">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="AP82" t="n">
         <v>30</v>
       </c>
       <c r="AQ82" t="n">
-        <v>85.40000000000001</v>
+        <v>78.2</v>
       </c>
       <c r="AR82" t="n">
         <v>100</v>
       </c>
       <c r="AS82" t="n">
-        <v>85.40000000000001</v>
+        <v>78.2</v>
       </c>
       <c r="AT82" t="inlineStr">
         <is>
@@ -16810,19 +16810,19 @@
         <v>50</v>
       </c>
       <c r="AO83" t="n">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="AP83" t="n">
         <v>30</v>
       </c>
       <c r="AQ83" t="n">
-        <v>53.8</v>
+        <v>49</v>
       </c>
       <c r="AR83" t="n">
         <v>100</v>
       </c>
       <c r="AS83" t="n">
-        <v>53.8</v>
+        <v>49</v>
       </c>
       <c r="AT83" t="inlineStr">
         <is>
@@ -17006,22 +17006,22 @@
         <v>5</v>
       </c>
       <c r="AN84" t="n">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="AO84" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="AP84" t="n">
         <v>30</v>
       </c>
       <c r="AQ84" t="n">
-        <v>77.59999999999999</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="AR84" t="n">
         <v>100</v>
       </c>
       <c r="AS84" t="n">
-        <v>77.59999999999999</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="AT84" t="inlineStr">
         <is>
@@ -17205,22 +17205,22 @@
         <v>5</v>
       </c>
       <c r="AN85" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO85" t="n">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="AP85" t="n">
         <v>30</v>
       </c>
       <c r="AQ85" t="n">
-        <v>84.8</v>
+        <v>78.2</v>
       </c>
       <c r="AR85" t="n">
         <v>100</v>
       </c>
       <c r="AS85" t="n">
-        <v>84.8</v>
+        <v>78.2</v>
       </c>
       <c r="AT85" t="inlineStr">
         <is>
@@ -17407,19 +17407,19 @@
         <v>80</v>
       </c>
       <c r="AO86" t="n">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="AP86" t="n">
         <v>30</v>
       </c>
       <c r="AQ86" t="n">
-        <v>60.8</v>
+        <v>58</v>
       </c>
       <c r="AR86" t="n">
         <v>100</v>
       </c>
       <c r="AS86" t="n">
-        <v>60.8</v>
+        <v>58</v>
       </c>
       <c r="AT86" t="inlineStr">
         <is>
@@ -17606,19 +17606,19 @@
         <v>80</v>
       </c>
       <c r="AO87" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="AP87" t="n">
         <v>30</v>
       </c>
       <c r="AQ87" t="n">
-        <v>48.4</v>
+        <v>44.8</v>
       </c>
       <c r="AR87" t="n">
         <v>100</v>
       </c>
       <c r="AS87" t="n">
-        <v>48.4</v>
+        <v>44.8</v>
       </c>
       <c r="AT87" t="inlineStr">
         <is>
@@ -17798,22 +17798,22 @@
         <v>5</v>
       </c>
       <c r="AN88" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO88" t="n">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="AP88" t="n">
         <v>30</v>
       </c>
       <c r="AQ88" t="n">
-        <v>85.2</v>
+        <v>78.2</v>
       </c>
       <c r="AR88" t="n">
         <v>100</v>
       </c>
       <c r="AS88" t="n">
-        <v>85.2</v>
+        <v>78.2</v>
       </c>
       <c r="AT88" t="inlineStr">
         <is>
@@ -17996,19 +17996,19 @@
         <v>80</v>
       </c>
       <c r="AO89" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="AP89" t="n">
         <v>30</v>
       </c>
       <c r="AQ89" t="n">
-        <v>48.4</v>
+        <v>44.8</v>
       </c>
       <c r="AR89" t="n">
         <v>100</v>
       </c>
       <c r="AS89" t="n">
-        <v>48.4</v>
+        <v>44.8</v>
       </c>
       <c r="AT89" t="inlineStr">
         <is>
@@ -18192,22 +18192,22 @@
         <v>5</v>
       </c>
       <c r="AN90" t="n">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="AO90" t="n">
-        <v>100</v>
+        <v>76</v>
       </c>
       <c r="AP90" t="n">
         <v>30</v>
       </c>
       <c r="AQ90" t="n">
-        <v>73.40000000000001</v>
+        <v>61.4</v>
       </c>
       <c r="AR90" t="n">
         <v>100</v>
       </c>
       <c r="AS90" t="n">
-        <v>73.40000000000001</v>
+        <v>61.4</v>
       </c>
       <c r="AT90" t="inlineStr">
         <is>
@@ -18391,22 +18391,22 @@
         <v>5</v>
       </c>
       <c r="AN91" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO91" t="n">
-        <v>93</v>
+        <v>62</v>
       </c>
       <c r="AP91" t="n">
         <v>30</v>
       </c>
       <c r="AQ91" t="n">
-        <v>83.2</v>
+        <v>67.8</v>
       </c>
       <c r="AR91" t="n">
         <v>100</v>
       </c>
       <c r="AS91" t="n">
-        <v>83.2</v>
+        <v>67.8</v>
       </c>
       <c r="AT91" t="inlineStr">
         <is>
@@ -18586,22 +18586,22 @@
         <v>5</v>
       </c>
       <c r="AN92" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO92" t="n">
-        <v>100</v>
+        <v>62</v>
       </c>
       <c r="AP92" t="n">
         <v>30</v>
       </c>
       <c r="AQ92" t="n">
-        <v>86</v>
+        <v>67.8</v>
       </c>
       <c r="AR92" t="n">
         <v>100</v>
       </c>
       <c r="AS92" t="n">
-        <v>86</v>
+        <v>67.8</v>
       </c>
       <c r="AT92" t="inlineStr">
         <is>
@@ -18781,22 +18781,22 @@
         <v>5</v>
       </c>
       <c r="AN93" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO93" t="n">
-        <v>98</v>
+        <v>76</v>
       </c>
       <c r="AP93" t="n">
         <v>30</v>
       </c>
       <c r="AQ93" t="n">
-        <v>85.2</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="AR93" t="n">
         <v>100</v>
       </c>
       <c r="AS93" t="n">
-        <v>85.2</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="AT93" t="inlineStr">
         <is>
@@ -18980,22 +18980,22 @@
         <v>5</v>
       </c>
       <c r="AN94" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AO94" t="n">
-        <v>53</v>
+        <v>28</v>
       </c>
       <c r="AP94" t="n">
         <v>30</v>
       </c>
       <c r="AQ94" t="n">
-        <v>67.2</v>
+        <v>51.2</v>
       </c>
       <c r="AR94" t="n">
         <v>100</v>
       </c>
       <c r="AS94" t="n">
-        <v>67.2</v>
+        <v>51.2</v>
       </c>
       <c r="AT94" t="inlineStr">
         <is>
@@ -19179,22 +19179,22 @@
         <v>5</v>
       </c>
       <c r="AN95" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AO95" t="n">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="AP95" t="n">
         <v>30</v>
       </c>
       <c r="AQ95" t="n">
-        <v>58.4</v>
+        <v>44.8</v>
       </c>
       <c r="AR95" t="n">
         <v>100</v>
       </c>
       <c r="AS95" t="n">
-        <v>58.4</v>
+        <v>44.8</v>
       </c>
       <c r="AT95" t="inlineStr">
         <is>
@@ -19377,19 +19377,19 @@
         <v>90</v>
       </c>
       <c r="AO96" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="AP96" t="n">
         <v>30</v>
       </c>
       <c r="AQ96" t="n">
-        <v>56.6</v>
+        <v>54.2</v>
       </c>
       <c r="AR96" t="n">
         <v>100</v>
       </c>
       <c r="AS96" t="n">
-        <v>56.6</v>
+        <v>54.2</v>
       </c>
       <c r="AT96" t="inlineStr">
         <is>
@@ -19573,22 +19573,22 @@
         <v>5</v>
       </c>
       <c r="AN97" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO97" t="n">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="AP97" t="n">
         <v>30</v>
       </c>
       <c r="AQ97" t="n">
-        <v>86</v>
+        <v>78.2</v>
       </c>
       <c r="AR97" t="n">
         <v>100</v>
       </c>
       <c r="AS97" t="n">
-        <v>86</v>
+        <v>78.2</v>
       </c>
       <c r="AT97" t="inlineStr">
         <is>
@@ -19779,19 +19779,19 @@
         <v>80</v>
       </c>
       <c r="AO98" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="AP98" t="n">
         <v>30</v>
       </c>
       <c r="AQ98" t="n">
-        <v>55.2</v>
+        <v>51.2</v>
       </c>
       <c r="AR98" t="n">
         <v>100</v>
       </c>
       <c r="AS98" t="n">
-        <v>55.2</v>
+        <v>51.2</v>
       </c>
       <c r="AT98" t="inlineStr">
         <is>
@@ -19975,22 +19975,22 @@
         <v>5</v>
       </c>
       <c r="AN99" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO99" t="n">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="AP99" t="n">
         <v>30</v>
       </c>
       <c r="AQ99" t="n">
-        <v>67.59999999999999</v>
+        <v>61</v>
       </c>
       <c r="AR99" t="n">
         <v>100</v>
       </c>
       <c r="AS99" t="n">
-        <v>67.59999999999999</v>
+        <v>61</v>
       </c>
       <c r="AT99" t="inlineStr">
         <is>
@@ -20177,19 +20177,19 @@
         <v>50</v>
       </c>
       <c r="AO100" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="AP100" t="n">
         <v>30</v>
       </c>
       <c r="AQ100" t="n">
-        <v>44.6</v>
+        <v>42.2</v>
       </c>
       <c r="AR100" t="n">
         <v>100</v>
       </c>
       <c r="AS100" t="n">
-        <v>44.6</v>
+        <v>42.2</v>
       </c>
       <c r="AT100" t="inlineStr">
         <is>
@@ -20376,19 +20376,19 @@
         <v>90</v>
       </c>
       <c r="AO101" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="AP101" t="n">
         <v>30</v>
       </c>
       <c r="AQ101" t="n">
-        <v>51.4</v>
+        <v>47.8</v>
       </c>
       <c r="AR101" t="n">
         <v>100</v>
       </c>
       <c r="AS101" t="n">
-        <v>51.4</v>
+        <v>47.8</v>
       </c>
       <c r="AT101" t="inlineStr">
         <is>
@@ -20575,19 +20575,19 @@
         <v>80</v>
       </c>
       <c r="AO102" t="n">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="AP102" t="n">
         <v>30</v>
       </c>
       <c r="AQ102" t="n">
-        <v>80</v>
+        <v>75.2</v>
       </c>
       <c r="AR102" t="n">
         <v>100</v>
       </c>
       <c r="AS102" t="n">
-        <v>80</v>
+        <v>75.2</v>
       </c>
       <c r="AT102" t="inlineStr">
         <is>
@@ -20767,7 +20767,7 @@
         <v>5</v>
       </c>
       <c r="AN103" t="n">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="AO103" t="n">
         <v>45</v>
@@ -20776,13 +20776,13 @@
         <v>30</v>
       </c>
       <c r="AQ103" t="n">
-        <v>60.4</v>
+        <v>58</v>
       </c>
       <c r="AR103" t="n">
         <v>100</v>
       </c>
       <c r="AS103" t="n">
-        <v>60.4</v>
+        <v>58</v>
       </c>
       <c r="AT103" t="inlineStr">
         <is>
@@ -20966,22 +20966,22 @@
         <v>5</v>
       </c>
       <c r="AN104" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="AO104" t="n">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="AP104" t="n">
         <v>30</v>
       </c>
       <c r="AQ104" t="n">
-        <v>58.5</v>
+        <v>51.2</v>
       </c>
       <c r="AR104" t="n">
         <v>100</v>
       </c>
       <c r="AS104" t="n">
-        <v>58.5</v>
+        <v>51.2</v>
       </c>
       <c r="AT104" t="inlineStr">
         <is>
@@ -21165,22 +21165,22 @@
         <v>5</v>
       </c>
       <c r="AN105" t="n">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="AO105" t="n">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="AP105" t="n">
         <v>30</v>
       </c>
       <c r="AQ105" t="n">
-        <v>76.40000000000001</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="AR105" t="n">
         <v>100</v>
       </c>
       <c r="AS105" t="n">
-        <v>76.40000000000001</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="AT105" t="inlineStr">
         <is>
@@ -21360,7 +21360,7 @@
         <v>5</v>
       </c>
       <c r="AN106" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AO106" t="n">
         <v>28</v>
@@ -21369,13 +21369,13 @@
         <v>30</v>
       </c>
       <c r="AQ106" t="n">
-        <v>56.6</v>
+        <v>54.2</v>
       </c>
       <c r="AR106" t="n">
         <v>100</v>
       </c>
       <c r="AS106" t="n">
-        <v>56.6</v>
+        <v>54.2</v>
       </c>
       <c r="AT106" t="inlineStr">
         <is>
@@ -21559,22 +21559,22 @@
         <v>5</v>
       </c>
       <c r="AN107" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="AO107" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="AP107" t="n">
         <v>30</v>
       </c>
       <c r="AQ107" t="n">
-        <v>67.40000000000001</v>
+        <v>61</v>
       </c>
       <c r="AR107" t="n">
         <v>100</v>
       </c>
       <c r="AS107" t="n">
-        <v>67.40000000000001</v>
+        <v>61</v>
       </c>
       <c r="AT107" t="inlineStr">
         <is>
@@ -21758,22 +21758,22 @@
         <v>5</v>
       </c>
       <c r="AN108" t="n">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="AO108" t="n">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="AP108" t="n">
         <v>30</v>
       </c>
       <c r="AQ108" t="n">
-        <v>50.6</v>
+        <v>42.2</v>
       </c>
       <c r="AR108" t="n">
         <v>100</v>
       </c>
       <c r="AS108" t="n">
-        <v>50.6</v>
+        <v>42.2</v>
       </c>
       <c r="AT108" t="inlineStr">
         <is>
@@ -21956,19 +21956,19 @@
         <v>80</v>
       </c>
       <c r="AO109" t="n">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="AP109" t="n">
         <v>30</v>
       </c>
       <c r="AQ109" t="n">
-        <v>54.8</v>
+        <v>51.2</v>
       </c>
       <c r="AR109" t="n">
         <v>100</v>
       </c>
       <c r="AS109" t="n">
-        <v>54.8</v>
+        <v>51.2</v>
       </c>
       <c r="AT109" t="inlineStr">
         <is>
@@ -22155,19 +22155,19 @@
         <v>80</v>
       </c>
       <c r="AO110" t="n">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="AP110" t="n">
         <v>30</v>
       </c>
       <c r="AQ110" t="n">
-        <v>56.8</v>
+        <v>51.2</v>
       </c>
       <c r="AR110" t="n">
         <v>100</v>
       </c>
       <c r="AS110" t="n">
-        <v>56.8</v>
+        <v>51.2</v>
       </c>
       <c r="AT110" t="inlineStr">
         <is>
@@ -22351,22 +22351,22 @@
         <v>5</v>
       </c>
       <c r="AN111" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AO111" t="n">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="AP111" t="n">
         <v>30</v>
       </c>
       <c r="AQ111" t="n">
-        <v>86</v>
+        <v>78.2</v>
       </c>
       <c r="AR111" t="n">
         <v>100</v>
       </c>
       <c r="AS111" t="n">
-        <v>86</v>
+        <v>78.2</v>
       </c>
       <c r="AT111" t="inlineStr">
         <is>
@@ -22553,19 +22553,19 @@
         <v>90</v>
       </c>
       <c r="AO112" t="n">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="AP112" t="n">
         <v>30</v>
       </c>
       <c r="AQ112" t="n">
-        <v>59.8</v>
+        <v>54.2</v>
       </c>
       <c r="AR112" t="n">
         <v>100</v>
       </c>
       <c r="AS112" t="n">
-        <v>59.8</v>
+        <v>54.2</v>
       </c>
       <c r="AT112" t="inlineStr">
         <is>
@@ -22749,22 +22749,22 @@
         <v>5</v>
       </c>
       <c r="AN113" t="n">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="AO113" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="AP113" t="n">
         <v>30</v>
       </c>
       <c r="AQ113" t="n">
-        <v>62.4</v>
+        <v>58</v>
       </c>
       <c r="AR113" t="n">
         <v>100</v>
       </c>
       <c r="AS113" t="n">
-        <v>62.4</v>
+        <v>58</v>
       </c>
       <c r="AT113" t="inlineStr">
         <is>
@@ -22951,19 +22951,19 @@
         <v>90</v>
       </c>
       <c r="AO114" t="n">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="AP114" t="n">
         <v>30</v>
       </c>
       <c r="AQ114" t="n">
-        <v>83</v>
+        <v>78.2</v>
       </c>
       <c r="AR114" t="n">
         <v>100</v>
       </c>
       <c r="AS114" t="n">
-        <v>83</v>
+        <v>78.2</v>
       </c>
       <c r="AT114" t="inlineStr">
         <is>
@@ -23151,22 +23151,22 @@
         <v>5</v>
       </c>
       <c r="AN115" t="n">
+        <v>80</v>
+      </c>
+      <c r="AO115" t="n">
         <v>88</v>
-      </c>
-      <c r="AO115" t="n">
-        <v>96</v>
       </c>
       <c r="AP115" t="n">
         <v>30</v>
       </c>
       <c r="AQ115" t="n">
-        <v>80.8</v>
+        <v>75.2</v>
       </c>
       <c r="AR115" t="n">
         <v>100</v>
       </c>
       <c r="AS115" t="n">
-        <v>80.8</v>
+        <v>75.2</v>
       </c>
       <c r="AT115" t="inlineStr">
         <is>
@@ -23354,7 +23354,7 @@
         <v>5</v>
       </c>
       <c r="AN116" t="n">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="AO116" t="n">
         <v>62</v>
@@ -23363,13 +23363,13 @@
         <v>30</v>
       </c>
       <c r="AQ116" t="n">
-        <v>60.6</v>
+        <v>55.8</v>
       </c>
       <c r="AR116" t="n">
         <v>100</v>
       </c>
       <c r="AS116" t="n">
-        <v>60.6</v>
+        <v>55.8</v>
       </c>
       <c r="AT116" t="inlineStr">
         <is>
@@ -23553,7 +23553,7 @@
         <v>5</v>
       </c>
       <c r="AN117" t="n">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="AO117" t="n">
         <v>88</v>
@@ -23562,13 +23562,13 @@
         <v>30</v>
       </c>
       <c r="AQ117" t="n">
-        <v>68.59999999999999</v>
+        <v>66.2</v>
       </c>
       <c r="AR117" t="n">
         <v>100</v>
       </c>
       <c r="AS117" t="n">
-        <v>68.59999999999999</v>
+        <v>66.2</v>
       </c>
       <c r="AT117" t="inlineStr">
         <is>
@@ -23752,22 +23752,22 @@
         <v>5</v>
       </c>
       <c r="AN118" t="n">
+        <v>80</v>
+      </c>
+      <c r="AO118" t="n">
         <v>88</v>
-      </c>
-      <c r="AO118" t="n">
-        <v>100</v>
       </c>
       <c r="AP118" t="n">
         <v>30</v>
       </c>
       <c r="AQ118" t="n">
-        <v>82.40000000000001</v>
+        <v>75.2</v>
       </c>
       <c r="AR118" t="n">
         <v>100</v>
       </c>
       <c r="AS118" t="n">
-        <v>82.40000000000001</v>
+        <v>75.2</v>
       </c>
       <c r="AT118" t="inlineStr">
         <is>
@@ -23954,19 +23954,19 @@
         <v>80</v>
       </c>
       <c r="AO119" t="n">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="AP119" t="n">
         <v>30</v>
       </c>
       <c r="AQ119" t="n">
-        <v>73.59999999999999</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="AR119" t="n">
         <v>100</v>
       </c>
       <c r="AS119" t="n">
-        <v>73.59999999999999</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="AT119" t="inlineStr">
         <is>
@@ -24153,19 +24153,19 @@
         <v>90</v>
       </c>
       <c r="AO120" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AP120" t="n">
         <v>30</v>
       </c>
       <c r="AQ120" t="n">
-        <v>47.4</v>
+        <v>47.8</v>
       </c>
       <c r="AR120" t="n">
         <v>100</v>
       </c>
       <c r="AS120" t="n">
-        <v>47.4</v>
+        <v>47.8</v>
       </c>
       <c r="AT120" t="inlineStr">
         <is>

</xml_diff>